<commit_message>
Complete final accessibility audit and capstone documentation
</commit_message>
<xml_diff>
--- a/docs/GoalBridge_Finance_Verification.xlsx
+++ b/docs/GoalBridge_Finance_Verification.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop Data 4 Aug 2026\FPA\AI\Capstone project 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319BA06D-D921-4E26-85F9-BAF3FC744BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D9EE96-A343-4BC8-8E38-2938C0A7B036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{87694B63-E9E9-4ED1-A661-B1A84B642EB3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{87694B63-E9E9-4ED1-A661-B1A84B642EB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Calculation Assumptions" sheetId="3" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId2"/>
+    <sheet name="Defect Sheet" sheetId="4" r:id="rId2"/>
+    <sheet name="Audhit Trail" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="Annual_Infaltion_Rate">'Calculation Assumptions'!$B$5</definedName>
@@ -55,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="104">
   <si>
     <t>Goal Amount Today</t>
   </si>
@@ -109,6 +110,371 @@
   </si>
   <si>
     <t>Cells B3:B7 contain the user-input assumptions. Cells B8:B16 contain calculated values/formulas and should not be manually entered.</t>
+  </si>
+  <si>
+    <t>Defect ID</t>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>DEF01</t>
+  </si>
+  <si>
+    <t>Goal Name containing only spaces bypasses validation</t>
+  </si>
+  <si>
+    <t>User can submit an apparently blank goal name, so required-field validation is incomplete</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>DEF02</t>
+  </si>
+  <si>
+    <t>Validation messages are inconsistent in wording, grammar, and source</t>
+  </si>
+  <si>
+    <t>Low / UX</t>
+  </si>
+  <si>
+    <t>Expected Behaviour</t>
+  </si>
+  <si>
+    <t>trim whitespace before validating. After trimming, an all-space value should be treated as blank and show:</t>
+  </si>
+  <si>
+    <t>Expcted Output</t>
+  </si>
+  <si>
+    <t>Error Messasge:  "Enter a goal name."</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">First-time users receive a mixture of custom messages and browser-native messages, some of which are unclear or inconsistent.
+Current Messsage are as below:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Current messages include:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+“Enter a goal name”
+“goal Amount must be greater than zero”
+“Value must be greater than or equal to 0.01”
+“Enter Zero or Positive number”
+“Please fill in this field”
+“years to goal must be positive number”
+“Value must be greater than or equal to 1”
+“Years to goal must be Positive or Whole number”
+“Enter Zero or Positive value”
+“enter value no greater than 100”</t>
+    </r>
+  </si>
+  <si>
+    <t>Proposed Standard message</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Recommended message</t>
+  </si>
+  <si>
+    <t>Goal Name blank/spaces</t>
+  </si>
+  <si>
+    <t>Enter a goal name.</t>
+  </si>
+  <si>
+    <t>Goal Amount blank</t>
+  </si>
+  <si>
+    <t>Enter the goal amount.</t>
+  </si>
+  <si>
+    <t>Goal Amount ≤ 0</t>
+  </si>
+  <si>
+    <t>Enter a goal amount greater than ₹0.</t>
+  </si>
+  <si>
+    <t>Current Savings blank</t>
+  </si>
+  <si>
+    <t>Enter current savings. Use 0 if you have no savings yet.</t>
+  </si>
+  <si>
+    <t>Current Savings &lt; 0</t>
+  </si>
+  <si>
+    <t>Enter zero or a positive amount.</t>
+  </si>
+  <si>
+    <t>Years blank</t>
+  </si>
+  <si>
+    <t>Enter the number of years to your goal.</t>
+  </si>
+  <si>
+    <t>Years ≤ 0</t>
+  </si>
+  <si>
+    <t>Enter a positive whole number of years.</t>
+  </si>
+  <si>
+    <t>Years decimal</t>
+  </si>
+  <si>
+    <t>Enter a whole number of years.</t>
+  </si>
+  <si>
+    <t>Inflation blank</t>
+  </si>
+  <si>
+    <t>Enter an expected annual inflation rate.</t>
+  </si>
+  <si>
+    <t>Inflation &lt; 0</t>
+  </si>
+  <si>
+    <t>Enter zero or a positive inflation rate.</t>
+  </si>
+  <si>
+    <t>Inflation &gt; allowed maximum</t>
+  </si>
+  <si>
+    <t>Enter an inflation rate no greater than 100%.</t>
+  </si>
+  <si>
+    <t>Return blank</t>
+  </si>
+  <si>
+    <t>Enter an expected annual investment return.</t>
+  </si>
+  <si>
+    <t>Return &lt; 0</t>
+  </si>
+  <si>
+    <t>Enter zero or a positive investment return.</t>
+  </si>
+  <si>
+    <t>Return &gt; 100</t>
+  </si>
+  <si>
+    <t>Enter an investment return no greater than 100%.</t>
+  </si>
+  <si>
+    <t>Messages should have consistnet wordings</t>
+  </si>
+  <si>
+    <t>refer: Propsoed Messages</t>
+  </si>
+  <si>
+    <t>Defect</t>
+  </si>
+  <si>
+    <t>Before</t>
+  </si>
+  <si>
+    <t>Fix</t>
+  </si>
+  <si>
+    <t>Retest</t>
+  </si>
+  <si>
+    <t>Spaces-only Goal Name bypassed validation</t>
+  </si>
+  <si>
+    <t>Trim input before validating</t>
+  </si>
+  <si>
+    <t>Spaces-only input now blocked</t>
+  </si>
+  <si>
+    <t>Validation wording inconsistent/browser-dependent</t>
+  </si>
+  <si>
+    <t>Standardized custom validation messages</t>
+  </si>
+  <si>
+    <t>Invalid inputs now show consistent messages</t>
+  </si>
+  <si>
+    <t>Regression</t>
+  </si>
+  <si>
+    <t>Finance engine could potentially be affected by JS changes</t>
+  </si>
+  <si>
+    <t>Automated regression suite</t>
+  </si>
+  <si>
+    <t>9/9 PASS</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Closed - Pass</t>
+  </si>
+  <si>
+    <r>
+      <t>Regression Testing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Following validation changes, the automated Vitest finance suite was rerun. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>All 9 tests passed (9/9)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, confirming that the validation changes did not alter the verified financial calculation engine.</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Valid boundary cases were manually confirmed:</t>
+  </si>
+  <si>
+    <t>3. Current Savings = 0, Inflation = 0%, and Expected Return = 0% remained valid after the changes.</t>
+  </si>
+  <si>
+    <t>Evidence</t>
+  </si>
+  <si>
+    <t>evidence\DEF01 Goal Name contain only Spaces.png</t>
+  </si>
+  <si>
+    <t>evidence\DEF02 Message Consistency.png</t>
+  </si>
+  <si>
+    <t>Accessibility audit status</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <r>
+      <t>A11Y-01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Keyboard navigation &amp; visible focus</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>A11Y-02</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 200% zoom/reflow</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>A11Y-03</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Chrome Lighthouse Accessibility</t>
+    </r>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>evidence\A11Y_01_keyboard_focus.png</t>
+  </si>
+  <si>
+    <t>evidence\A11Y-02 — 200% Zoom.png</t>
+  </si>
+  <si>
+    <t>evidence\A11Y-03 — Lighthouse Accessibility.png</t>
+  </si>
+  <si>
+    <t>All interactive controls in the final production application were reachable using keyboard-only navigation. Forward and reverse tab navigation worked logically, visible focus indicators were present, controls could be activated using expected keyboard actions, and no keyboard trap was observed</t>
+  </si>
+  <si>
+    <t>No overlap, breakage or loss of functionality; screenshot captured.</t>
+  </si>
+  <si>
+    <t>Environment: Production Vercel deployment / Google Chrome Lighthouse
+Automated accessibility audit reported no scored accessibility failures. Lighthouse's additional manual-check items were addressed separately through manual accessibility testing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 100/100 PASS</t>
   </si>
 </sst>
 </file>
@@ -117,9 +483,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    <numFmt numFmtId="169" formatCode="0.0000%"/>
+    <numFmt numFmtId="165" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +521,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -170,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -241,11 +623,58 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
@@ -293,24 +722,79 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -709,7 +1193,7 @@
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="13">
         <f>years_to_Goal*12</f>
         <v>120</v>
       </c>
@@ -718,7 +1202,7 @@
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="15">
+      <c r="B9" s="14">
         <f>(1+Expected_Investment_Return)^(1/12)-1</f>
         <v>7.9741404289037643E-3</v>
       </c>
@@ -727,13 +1211,13 @@
       <c r="A10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="16"/>
+      <c r="B10" s="15"/>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="16">
         <f>Goal_amout_today*(1+Annual_Infaltion_Rate)^years_to_Goal</f>
         <v>2149017.2358514257</v>
       </c>
@@ -742,7 +1226,7 @@
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="16">
         <f>current_Saving*(1+Expected_Investment_Return)^years_to_Goal</f>
         <v>389061.36901500029</v>
       </c>
@@ -751,7 +1235,7 @@
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="16">
         <f>MAX(0,Goal_Value-fund_Value_of_Current_Savings)</f>
         <v>1759955.8668364254</v>
       </c>
@@ -760,7 +1244,7 @@
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="17">
+      <c r="B14" s="16">
         <f>IF(effective_monthly_rate=0,Funding_Gap/Number_of_Months,Funding_Gap*effective_monthly_rate/((1+effective_monthly_rate)^Number_of_Months-1))</f>
         <v>8805.7735689278506</v>
       </c>
@@ -769,7 +1253,7 @@
       <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="17">
+      <c r="B15" s="16">
         <f>Required_Monthly_contribution*Number_of_Months</f>
         <v>1056692.828271342</v>
       </c>
@@ -778,7 +1262,7 @@
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="17">
+      <c r="B16" s="16">
         <f>Funding_Gap-Total_Monhtly_contributions</f>
         <v>703263.03856508341</v>
       </c>
@@ -787,10 +1271,10 @@
       <c r="B17" s="12"/>
     </row>
     <row r="18" spans="1:2" ht="45.6" customHeight="1">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="13"/>
+      <c r="B18" s="28"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
@@ -803,9 +1287,395 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD46A69-7A9F-4FD4-8084-13C5A2007021}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24.109375" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="5" max="5" width="28.21875" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="57.6">
+      <c r="A2" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="244.8">
+      <c r="A3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="30"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8">
+      <c r="A10" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="28.8">
+      <c r="A15" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28.8">
+      <c r="A17" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="28.8">
+      <c r="A18" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28.8">
+      <c r="A19" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28.8">
+      <c r="A20" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+    </row>
+    <row r="23" spans="1:4" ht="31.8" customHeight="1">
+      <c r="A23" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="31" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A22:D22"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F3" location="'Defect Sheet'!A5" display="refer: Propsoed Messages" xr:uid="{3F76CCB0-9416-4ADD-9D49-B21E1964CF51}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75550105-EC68-4CC6-B77F-75C73595F24C}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36.21875" customWidth="1"/>
+    <col min="2" max="2" width="44.44140625" customWidth="1"/>
+    <col min="3" max="3" width="41.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.8">
+      <c r="A4" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="18">
+      <c r="A6" s="26" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="86.4">
+      <c r="A9" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28.8">
+      <c r="A10" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="100.8">
+      <c r="A11" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>